<commit_message>
📊 Línea 141 actualizada
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-01-10.xlsx
+++ b/data/horarios-141-2026-01-10.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP1912" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP1912-215" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6203-6173" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LP1912" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LP1912-215" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="6203-6173" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,14 +441,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:52:16</t>
+          <t>Actualizado: 14:10:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>16 únicos (por Identificador)</t>
         </is>
       </c>
     </row>
@@ -483,6 +483,11 @@
           <t>CodigoColectivo</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Identificador</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -509,6 +514,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -535,6 +541,7 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -561,6 +568,7 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -587,6 +595,7 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -613,6 +622,7 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -639,6 +649,7 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -665,6 +676,7 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -691,6 +703,7 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -717,6 +730,7 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -743,6 +757,7 @@
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -769,6 +784,7 @@
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -795,6 +811,7 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -821,6 +838,88 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:10:09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:10:09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:10:09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:49</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>39</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -833,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,14 +945,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:52:16</t>
+          <t>Actualizado: 14:10:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>1 únicos (por Identificador)</t>
         </is>
       </c>
     </row>
@@ -888,6 +987,11 @@
           <t>CodigoColectivo</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Identificador</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -914,6 +1018,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -926,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -939,14 +1044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:52:16</t>
+          <t>Actualizado: 14:10:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>4 únicos (por Identificador)</t>
         </is>
       </c>
     </row>
@@ -981,6 +1086,11 @@
           <t>CodigoColectivo</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Identificador</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1007,6 +1117,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1033,6 +1144,7 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1059,6 +1171,34 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>